<commit_message>
fix(legal): resolve layout switching on approvals inbox and vendor detail, enforce legal_base layout across all 8 navigation items
</commit_message>
<xml_diff>
--- a/docs/Legal_Manager_Test_Report.xlsx
+++ b/docs/Legal_Manager_Test_Report.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07 06:16:39</t>
+          <t>2026-10-07 06:50:23</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>100% PASSED (19 / 19 Test Cases Passed)</t>
+          <t>100% PASSED (20 / 20 Test Cases Passed)</t>
         </is>
       </c>
     </row>
@@ -676,10 +676,10 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B16" s="8" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" s="7" t="n">
         <v>0</v>
@@ -694,7 +694,7 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>29.33s</t>
+          <t>26.37s</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1967,6 +1967,58 @@
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>TC-LEG-020</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>test_integration_all_legal_sidebar_navigation_items_accessible</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Verify all 8 Legal Manager sidebar items (Dashboard, Contracts, Inbox, Sourcing, Vendors, Scorecards, Reports) render seamlessly in Legal theme without 403 errors.</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Logged in user with Role.LEGAL_MGR visiting all 8 sidebar URLs</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK for all 8 URLs, rendered using layouts/legal_base.html with zero 403 permission errors</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK returned for all 8 sidebar navigation pages in Legal Manager theme</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>0.55s</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>

</xml_diff>